<commit_message>
Define continuidade, público, barreiras e impacto social do LendoJuntos
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -3071,12 +3071,28 @@
       </c>
     </row>
     <row r="2" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="40"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="42"/>
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Definição do formato de intervenção</t>
+        </is>
+      </c>
+      <c r="B2" s="41">
+        <v>46258</v>
+      </c>
+      <c r="C2" s="40" t="inlineStr">
+        <is>
+          <t>Alinhamento da continuidade do LendoJuntos como intervenção; delimitação do público, das barreiras e do impacto social.</t>
+        </is>
+      </c>
+      <c r="D2" s="42">
+        <v>2</v>
+      </c>
       <c r="E2" s="42"/>
-      <c r="F2" s="40"/>
+      <c r="F2" s="40" t="inlineStr">
+        <is>
+          <t>docs/semana-01-parte-1-intervencao.md</t>
+        </is>
+      </c>
       <c r="H2" s="16"/>
       <c r="I2" s="16"/>
       <c r="J2" s="16"/>

</xml_diff>

<commit_message>
Conclui estudo de acessibilidade e matriz WCAG 2.2 A/AA
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -3104,12 +3104,28 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="40"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="42"/>
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Pesquisa e estudo sobre o tema da causa ou cliente (leituras, visitas etc.)</t>
+        </is>
+      </c>
+      <c r="B3" s="41">
+        <v>46264</v>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>Estudo de acessibilidade digital e WCAG 2.2 A/AA; produção do fichamento e da matriz de 55 critérios aplicados às jornadas do LendoJuntos.</t>
+        </is>
+      </c>
+      <c r="D3" s="42">
+        <v>2</v>
+      </c>
       <c r="E3" s="42"/>
-      <c r="F3" s="40"/>
+      <c r="F3" s="40" t="inlineStr">
+        <is>
+          <t>docs/semana-01-parte-2-wcag.md</t>
+        </is>
+      </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
       <c r="J3" s="16"/>

</xml_diff>

<commit_message>
docs: adicionar relatório inicial e backlog priorizado da semana 3
- auditar a linha de base de acessibilidade nas nove telas e seis fluxos críticos
- priorizar 14 achados e duas validações técnicas com critérios de aceite
- preencher a Semana 3 na planilha de acessibilidade e tecnologias assistivas
- remover do cronograma as referências a validação e revisão com orientador
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leogu\OneDrive\Documentos\GitHub\lendojuntos\docs\academico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{27ED7794-3D1B-4606-B9AA-4E7BF49B9F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526CC143-1F35-4B12-B4D0-B37AFA27A1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,6 @@
     <sheet name="Leonardo Guilhon" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" forceFullCalc="1"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
   <si>
     <t>PROJETO:</t>
   </si>
@@ -150,6 +149,25 @@
   </si>
   <si>
     <t>Análise e Desenvolvimento de Sistemas</t>
+  </si>
+  <si>
+    <t>Alinhamento da continuidade do LendoJuntos como intervenção; delimitação do público, das barreiras e do impacto social.</t>
+  </si>
+  <si>
+    <t>docs/semana-01-parte-1-intervencao.md</t>
+  </si>
+  <si>
+    <t>Estudo de acessibilidade digital e WCAG 2.2 A/AA; produção do fichamento e da matriz de 55 critérios aplicados às jornadas do LendoJuntos.</t>
+  </si>
+  <si>
+    <t>docs/semana-01-parte-2-wcag.md</t>
+  </si>
+  <si>
+    <t>Auditoria da linha de base de acessibilidade do LendoJuntos; triagem dos 55 critérios WCAG 2.2 A/AA; consolidação de 14 achados e organização do backlog priorizado com critérios de aceite.</t>
+  </si>
+  <si>
+    <t>docs/semana-03-relatorio-inicial-auditoria.md
+docs/semana-03-backlog-priorizado-acessibilidade.md</t>
   </si>
 </sst>
 </file>
@@ -3070,28 +3088,22 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>Definição do formato de intervenção</t>
-        </is>
+    <row r="2" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" s="40" t="s">
+        <v>16</v>
       </c>
       <c r="B2" s="41">
         <v>46258</v>
       </c>
-      <c r="C2" s="40" t="inlineStr">
-        <is>
-          <t>Alinhamento da continuidade do LendoJuntos como intervenção; delimitação do público, das barreiras e do impacto social.</t>
-        </is>
+      <c r="C2" s="40" t="s">
+        <v>38</v>
       </c>
       <c r="D2" s="42">
         <v>2</v>
       </c>
       <c r="E2" s="42"/>
-      <c r="F2" s="40" t="inlineStr">
-        <is>
-          <t>docs/semana-01-parte-1-intervencao.md</t>
-        </is>
+      <c r="F2" s="40" t="s">
+        <v>39</v>
       </c>
       <c r="H2" s="16"/>
       <c r="I2" s="16"/>
@@ -3103,28 +3115,22 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="inlineStr">
-        <is>
-          <t>Pesquisa e estudo sobre o tema da causa ou cliente (leituras, visitas etc.)</t>
-        </is>
+    <row r="3" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+      <c r="A3" s="40" t="s">
+        <v>15</v>
       </c>
       <c r="B3" s="41">
         <v>46264</v>
       </c>
-      <c r="C3" s="40" t="inlineStr">
-        <is>
-          <t>Estudo de acessibilidade digital e WCAG 2.2 A/AA; produção do fichamento e da matriz de 55 critérios aplicados às jornadas do LendoJuntos.</t>
-        </is>
+      <c r="C3" s="40" t="s">
+        <v>40</v>
       </c>
       <c r="D3" s="42">
         <v>2</v>
       </c>
       <c r="E3" s="42"/>
-      <c r="F3" s="40" t="inlineStr">
-        <is>
-          <t>docs/semana-01-parte-2-wcag.md</t>
-        </is>
+      <c r="F3" s="40" t="s">
+        <v>41</v>
       </c>
       <c r="H3" s="16"/>
       <c r="I3" s="16"/>
@@ -3132,13 +3138,23 @@
       <c r="K3" s="16"/>
       <c r="L3" s="16"/>
     </row>
-    <row r="4" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="40"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="42"/>
+    <row r="4" spans="1:26" ht="72" x14ac:dyDescent="0.2">
+      <c r="A4" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="41">
+        <v>46277</v>
+      </c>
+      <c r="C4" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="42">
+        <v>4</v>
+      </c>
       <c r="E4" s="42"/>
-      <c r="F4" s="40"/>
+      <c r="F4" s="40" t="s">
+        <v>43</v>
+      </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" s="16"/>

</xml_diff>

<commit_message>
docs: concluir planejamento tecnico da semana 4
- definir padrões, ambiente, camadas e lotes do plano técnico de acessibilidade
- documentar fluxos, severidade, critérios de aceite e ciclo de reteste
- selecionar ferramentas manuais e automatizadas com seus limites
- registrar as 4 horas da semana na planilha acadêmica
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leogu\OneDrive\Documentos\GitHub\lendojuntos\docs\academico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526CC143-1F35-4B12-B4D0-B37AFA27A1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{763757FC-0C29-47B1-8B92-0685E6FC4CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>PROJETO:</t>
   </si>
@@ -168,6 +168,19 @@
   <si>
     <t>docs/semana-03-relatorio-inicial-auditoria.md
 docs/semana-03-backlog-priorizado-acessibilidade.md</t>
+  </si>
+  <si>
+    <t>Seleção e hierarquização de WCAG 2.2 A/AA, eMAG 3.1, WCAG-EM, WAI-ARIA APG e ferramentas manuais e automáticas; definição das camadas, do ambiente e dos lotes do plano técnico.</t>
+  </si>
+  <si>
+    <t>docs/semana-04-plano-tecnico-acessibilidade.md
+docs/semana-04-matriz-ferramentas-acessibilidade.md</t>
+  </si>
+  <si>
+    <t>Definição dos seis fluxos de teste, escala de severidade, prioridades, critérios de aceite, protocolos por modo de acesso e ciclo diagnosticar–corrigir–retestar.</t>
+  </si>
+  <si>
+    <t>docs/semana-04-metodologia-testes-acessibilidade.md</t>
   </si>
 </sst>
 </file>
@@ -360,7 +373,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -486,6 +499,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3161,26 +3177,48 @@
       <c r="K4" s="16"/>
       <c r="L4" s="16"/>
     </row>
-    <row r="5" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="40"/>
-      <c r="B5" s="41"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="42"/>
+    <row r="5" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+      <c r="A5" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="41">
+        <v>46284</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="42">
+        <v>2</v>
+      </c>
       <c r="E5" s="42"/>
-      <c r="F5" s="40"/>
+      <c r="F5" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="44"/>
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
       <c r="J5" s="16"/>
       <c r="K5" s="16"/>
       <c r="L5" s="16"/>
     </row>
-    <row r="6" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="40"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="42"/>
+    <row r="6" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+      <c r="A6" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="41">
+        <v>46284</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="42">
+        <v>2</v>
+      </c>
       <c r="E6" s="42"/>
-      <c r="F6" s="40"/>
+      <c r="F6" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="44"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="16"/>

</xml_diff>

<commit_message>
docs: concluir wireframes acessiveis da semana 5
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
   <si>
     <t>PROJETO:</t>
   </si>
@@ -181,6 +181,22 @@
   </si>
   <si>
     <t>docs/semana-04-metodologia-testes-acessibilidade.md</t>
+  </si>
+  <si>
+    <t>Estudo do eMAG 3.1 e de tecnologias assistivas; experimentos com teclado, NVDA, zoom/reflow e alto contraste; inventário das telas, dos estados e dos fluxos críticos do LendoJuntos.</t>
+  </si>
+  <si>
+    <t>docs/semana-02-checklist-emag.md
+docs/semana-02-notas-tecnologias-assistivas.md
+docs/semana-02-inventario-telas-fluxos.md
+docs/semana-02-experimento-browser.mjs</t>
+  </si>
+  <si>
+    <t>Criação dos wireframes acessíveis de baixa fidelidade para as nove telas e os padrões compartilhados; anotação dos seis fluxos críticos com landmarks, títulos, ordem de foco, formulários, cartões, menus, diálogos, estados e comportamento responsivo.</t>
+  </si>
+  <si>
+    <t>docs/semana-05-wireframes-acessiveis.md
+docs/semana-05-fluxos-anotados.md</t>
   </si>
 </sst>
 </file>
@@ -3156,20 +3172,20 @@
     </row>
     <row r="4" spans="1:26" ht="72" x14ac:dyDescent="0.2">
       <c r="A4" s="40" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B4" s="41">
-        <v>46277</v>
+        <v>46268</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D4" s="42">
         <v>4</v>
       </c>
       <c r="E4" s="42"/>
       <c r="F4" s="40" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
@@ -3179,20 +3195,20 @@
     </row>
     <row r="5" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A5" s="40" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B5" s="41">
-        <v>46284</v>
+        <v>46277</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D5" s="42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" s="42"/>
       <c r="F5" s="40" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G5" s="44"/>
       <c r="H5" s="16"/>
@@ -3203,20 +3219,20 @@
     </row>
     <row r="6" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="40" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="41">
         <v>46284</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D6" s="42">
         <v>2</v>
       </c>
       <c r="E6" s="42"/>
       <c r="F6" s="40" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G6" s="44"/>
       <c r="H6" s="16"/>
@@ -3226,12 +3242,22 @@
       <c r="L6" s="16"/>
     </row>
     <row r="7" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="40"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="42"/>
+      <c r="A7" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="41">
+        <v>46284</v>
+      </c>
+      <c r="C7" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="42">
+        <v>2</v>
+      </c>
       <c r="E7" s="42"/>
-      <c r="F7" s="40"/>
+      <c r="F7" s="40" t="s">
+        <v>47</v>
+      </c>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
@@ -3239,12 +3265,22 @@
       <c r="L7" s="16"/>
     </row>
     <row r="8" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="40"/>
-      <c r="B8" s="41"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="42"/>
+      <c r="A8" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="41">
+        <v>46293</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="42">
+        <v>4</v>
+      </c>
       <c r="E8" s="42"/>
-      <c r="F8" s="40"/>
+      <c r="F8" s="40" t="s">
+        <v>51</v>
+      </c>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
       <c r="J8" s="16"/>
@@ -3545,12 +3581,8 @@
       <c r="G31" s="16"/>
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
-      <c r="J31" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="K31" s="16">
-        <v>300</v>
-      </c>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
     </row>
     <row r="32" spans="1:12" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A32" s="32"/>
@@ -3577,6 +3609,12 @@
       <c r="E33" s="32"/>
       <c r="F33" s="32"/>
       <c r="G33" s="32"/>
+      <c r="J33" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="K33" s="32">
+        <v>300</v>
+      </c>
     </row>
     <row r="34" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="32"/>
@@ -3592,10 +3630,7 @@
       <c r="B35" s="35"/>
       <c r="C35" s="43"/>
       <c r="D35" s="43"/>
-      <c r="E35" s="43">
-        <f>SUM(E2:E33)</f>
-        <v>0</v>
-      </c>
+      <c r="E35" s="43"/>
       <c r="F35" s="32"/>
       <c r="G35" s="32"/>
     </row>
@@ -3604,7 +3639,10 @@
       <c r="B36" s="35"/>
       <c r="C36" s="32"/>
       <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
+      <c r="E36" s="32">
+        <f>SUM(E2:E34)</f>
+        <v>0</v>
+      </c>
       <c r="F36" s="32"/>
       <c r="G36" s="32"/>
     </row>

</xml_diff>

<commit_message>
docs: concluir prototipo acessivel da semana 6
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>PROJETO:</t>
   </si>
@@ -197,6 +197,15 @@
   <si>
     <t>docs/semana-05-wireframes-acessiveis.md
 docs/semana-05-fluxos-anotados.md</t>
+  </si>
+  <si>
+    <t>Conclusão do protótipo acessível de alta fidelidade para as nove telas; definição do guia visual e das especificações de contraste, foco, tipografia, estados, movimento e zoom/reflow; validação do protótipo em 1280, 640 e 320 CSS px.</t>
+  </si>
+  <si>
+    <t>docs/semana-06-prototipo-alta-fidelidade.md
+docs/semana-06-guia-visual-acessibilidade.md
+docs/semana-06-especificacoes-prototipo.md
+docs/prototipo-semana-06/</t>
   </si>
 </sst>
 </file>
@@ -3288,12 +3297,22 @@
       <c r="L8" s="16"/>
     </row>
     <row r="9" spans="1:26" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="40"/>
-      <c r="B9" s="41"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="42"/>
+      <c r="A9" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="41">
+        <v>46297</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="42">
+        <v>4</v>
+      </c>
       <c r="E9" s="42"/>
-      <c r="F9" s="40"/>
+      <c r="F9" s="40" t="s">
+        <v>53</v>
+      </c>
       <c r="H9" s="19"/>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>

</xml_diff>

<commit_message>
feat: concluir formularios acessiveis da semana 9
</commit_message>
<xml_diff>
--- a/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
+++ b/docs/academico/Leonardo Guilhon -  Acessibilidade e tecnologias assistivas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leogu\OneDrive\Documentos\GitHub\lendojuntos\docs\academico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1655F5EE-687A-4A87-B9EB-C352F4CC7773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4805116C-BB3A-4F22-BB5C-6A49A48C9735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="60">
   <si>
     <t>HORAS INVESTIDAS NO PROJETO POR ALUNO, EM CADA ETAPA (PREENCHIMENTO PELO ALUNO):</t>
   </si>
@@ -226,6 +226,17 @@
 docs/semana-08-validar-sobreposicoes.mjs
 frontend/src/components/Modal.tsx
 frontend/src/components/ActionMenu.tsx</t>
+  </si>
+  <si>
+    <t>Adequação dos formulários de login, cadastro e perfil: instruções, finalidade dos campos, validação com erros associados, foco para correção, anúncios de carregamento/erro/sucesso, preservação de dados e revisão do perfil antes da persistência; criação de roteiro automatizado e regressão dos lotes anteriores.</t>
+  </si>
+  <si>
+    <t>docs/semana-09-implementacao-formularios.md
+docs/semana-09-validar-formularios.mjs
+frontend/src/pages/LoginPage.tsx
+frontend/src/pages/RegisterPage.tsx
+frontend/src/pages/ProfilePage.tsx
+frontend/src/utils/formValidation.ts</t>
   </si>
 </sst>
 </file>
@@ -2042,7 +2053,7 @@
         <v>120</v>
       </c>
       <c r="C11" s="22">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D11" s="22"/>
       <c r="E11" s="22"/>
@@ -2104,7 +2115,7 @@
       </c>
       <c r="C14" s="39">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D14" s="30">
         <f t="shared" si="0"/>
@@ -3411,12 +3422,22 @@
       <c r="L11" s="16"/>
     </row>
     <row r="12" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="40"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="42"/>
+      <c r="A12" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="41">
+        <v>46321</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="42">
+        <v>5</v>
+      </c>
       <c r="E12" s="42"/>
-      <c r="F12" s="40"/>
+      <c r="F12" s="40" t="s">
+        <v>59</v>
+      </c>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
       <c r="J12" s="16"/>

</xml_diff>